<commit_message>
More progress with phenology model
</commit_message>
<xml_diff>
--- a/Prototypes/Lentil/CEData.xlsx
+++ b/Prototypes/Lentil/CEData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubRepos\ApsimX\Prototypes\Lentil\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99153353-16CD-465C-90B0-A78A85FDF3D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50F844CE-765C-4691-AA0E-642ADBCD8B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-5925" windowWidth="16440" windowHeight="28320" activeTab="2" xr2:uid="{A5017088-8F3F-41C2-9D3D-102B2E5948D4}"/>
+    <workbookView xWindow="-16320" yWindow="-5925" windowWidth="16440" windowHeight="28320" activeTab="1" xr2:uid="{A5017088-8F3F-41C2-9D3D-102B2E5948D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Roberts_etal_1988" sheetId="1" r:id="rId1"/>
@@ -72,9 +72,6 @@
   </si>
   <si>
     <t>ILL4349</t>
-  </si>
-  <si>
-    <t>Ethiopia</t>
   </si>
   <si>
     <t>Syrian</t>
@@ -240,6 +237,9 @@
   </si>
   <si>
     <t>Lentil.Phenology.StartFloweringTt</t>
+  </si>
+  <si>
+    <t>Ethiopian</t>
   </si>
 </sst>
 </file>
@@ -1234,7 +1234,7 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1243,25 +1243,25 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>53</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>54</v>
       </c>
-      <c r="G1" t="s">
-        <v>55</v>
-      </c>
       <c r="H1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" t="s">
         <v>50</v>
-      </c>
-      <c r="I1" t="s">
-        <v>35</v>
-      </c>
-      <c r="J1" t="s">
-        <v>51</v>
       </c>
       <c r="K1" t="s">
         <v>1</v>
@@ -1270,7 +1270,7 @@
         <v>2</v>
       </c>
       <c r="M1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -10656,7 +10656,7 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -10665,34 +10665,34 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" t="s">
         <v>53</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J1" t="s">
+        <v>59</v>
+      </c>
+      <c r="K1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L1" t="s">
         <v>61</v>
       </c>
-      <c r="G1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H1" t="s">
-        <v>63</v>
-      </c>
-      <c r="I1" t="s">
-        <v>59</v>
-      </c>
-      <c r="J1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>50</v>
-      </c>
-      <c r="L1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" t="s">
-        <v>51</v>
       </c>
       <c r="N1" t="s">
         <v>1</v>
@@ -10701,7 +10701,7 @@
         <v>2</v>
       </c>
       <c r="P1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -12086,10 +12086,10 @@
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin5oCFinalPp10hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin5oCFinalPp10hCvEthiopian</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>4</v>
@@ -12143,10 +12143,10 @@
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin5oCFinalPp10hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin5oCFinalPp10hCvEthiopian</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>4</v>
@@ -12200,10 +12200,10 @@
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin13oCFinalPp10hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin13oCFinalPp10hCvEthiopian</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>4</v>
@@ -12257,10 +12257,10 @@
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin13oCFinalPp10hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin13oCFinalPp10hCvEthiopian</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>4</v>
@@ -12314,10 +12314,10 @@
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin5oCFinalPp13hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin5oCFinalPp13hCvEthiopian</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>4</v>
@@ -12371,10 +12371,10 @@
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin13oCFinalPp13hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin13oCFinalPp13hCvEthiopian</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>4</v>
@@ -12428,10 +12428,10 @@
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin5oCFinalPp13hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin5oCFinalPp13hCvEthiopian</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>4</v>
@@ -12485,10 +12485,10 @@
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin13oCFinalPp13hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin13oCFinalPp13hCvEthiopian</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>4</v>
@@ -12542,10 +12542,10 @@
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin5oCFinalPp16hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin5oCFinalPp16hCvEthiopian</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>4</v>
@@ -12599,10 +12599,10 @@
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin13oCFinalPp16hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax18oCFinalTmin13oCFinalPp16hCvEthiopian</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>4</v>
@@ -12656,10 +12656,10 @@
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin5oCFinalPp16hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin5oCFinalPp16hCvEthiopian</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>4</v>
@@ -12713,10 +12713,10 @@
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin13oCFinalPp16hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat0FinalTmax28oCFinalTmin13oCFinalPp16hCvEthiopian</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
@@ -12770,10 +12770,10 @@
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin5oCFinalPp10hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin5oCFinalPp10hCvEthiopian</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>4</v>
@@ -12827,10 +12827,10 @@
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin5oCFinalPp10hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin5oCFinalPp10hCvEthiopian</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>4</v>
@@ -12885,10 +12885,10 @@
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin13oCFinalPp10hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin13oCFinalPp10hCvEthiopian</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>4</v>
@@ -12943,10 +12943,10 @@
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin13oCFinalPp10hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin13oCFinalPp10hCvEthiopian</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>4</v>
@@ -13001,10 +13001,10 @@
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin5oCFinalPp13hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin5oCFinalPp13hCvEthiopian</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>4</v>
@@ -13059,10 +13059,10 @@
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin13oCFinalPp13hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin13oCFinalPp13hCvEthiopian</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>4</v>
@@ -13117,10 +13117,10 @@
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin5oCFinalPp13hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin5oCFinalPp13hCvEthiopian</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>4</v>
@@ -13175,10 +13175,10 @@
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin13oCFinalPp13hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin13oCFinalPp13hCvEthiopian</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>4</v>
@@ -13233,10 +13233,10 @@
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin5oCFinalPp16hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin5oCFinalPp16hCvEthiopian</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>4</v>
@@ -13291,10 +13291,10 @@
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin13oCFinalPp16hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax18oCFinalTmin13oCFinalPp16hCvEthiopian</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>4</v>
@@ -13349,10 +13349,10 @@
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin5oCFinalPp16hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin5oCFinalPp16hCvEthiopian</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>4</v>
@@ -13407,10 +13407,10 @@
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" t="str">
         <f t="shared" si="4"/>
-        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin13oCFinalPp16hCvEthiopia</v>
+        <v>Summerfield1985InitT1oCDurat30FinalTmax28oCFinalTmin13oCFinalPp16hCvEthiopian</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>4</v>
@@ -14666,7 +14666,7 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -14675,25 +14675,25 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>53</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>54</v>
       </c>
-      <c r="G1" t="s">
-        <v>55</v>
-      </c>
       <c r="H1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" t="s">
         <v>50</v>
-      </c>
-      <c r="I1" t="s">
-        <v>58</v>
-      </c>
-      <c r="J1" t="s">
-        <v>51</v>
       </c>
       <c r="K1" t="s">
         <v>1</v>
@@ -14702,22 +14702,22 @@
         <v>2</v>
       </c>
       <c r="M1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="O1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="P1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q1" t="s">
         <v>47</v>
       </c>
-      <c r="Q1" t="s">
-        <v>48</v>
-      </c>
       <c r="R1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
@@ -14726,10 +14726,10 @@
         <v>Roberts1986Pp10to16hDurat45CvSyrian</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
       </c>
       <c r="D2" s="1">
         <v>10</v>
@@ -14765,7 +14765,7 @@
         <v>1478.5321100917445</v>
       </c>
       <c r="N2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O2">
         <f>F2*MIN(H2,I2)</f>
@@ -14790,10 +14790,10 @@
         <v>Roberts1986Pp10to16hDurat41CvSyrian</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
         <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
       </c>
       <c r="D3" s="1">
         <v>10</v>
@@ -14829,7 +14829,7 @@
         <v>1428.623853211009</v>
       </c>
       <c r="N3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O3">
         <f t="shared" ref="O3:O66" si="4">F3*MIN(H3,I3)</f>
@@ -14854,10 +14854,10 @@
         <v>Roberts1986Pp10to16hDurat37CvSyrian</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
         <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
       </c>
       <c r="D4" s="1">
         <v>10</v>
@@ -14893,7 +14893,7 @@
         <v>1335.045871559631</v>
       </c>
       <c r="N4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O4">
         <f t="shared" si="4"/>
@@ -14918,10 +14918,10 @@
         <v>Roberts1986Pp10to16hDurat33CvSyrian</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
         <v>10</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
       </c>
       <c r="D5" s="1">
         <v>10</v>
@@ -14957,7 +14957,7 @@
         <v>1241.4678899082564</v>
       </c>
       <c r="N5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="O5">
         <f t="shared" si="4"/>
@@ -14982,10 +14982,10 @@
         <v>Roberts1986Pp10to16hDurat29CvSyrian</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
         <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
       </c>
       <c r="D6" s="1">
         <v>10</v>
@@ -15021,7 +15021,7 @@
         <v>1122.9357798165133</v>
       </c>
       <c r="N6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="O6">
         <f t="shared" si="4"/>
@@ -15046,10 +15046,10 @@
         <v>Roberts1986Pp10to16hDurat25CvSyrian</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
         <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
       </c>
       <c r="D7" s="1">
         <v>10</v>
@@ -15085,7 +15085,7 @@
         <v>1066.7889908256873</v>
       </c>
       <c r="N7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O7">
         <f t="shared" si="4"/>
@@ -15110,10 +15110,10 @@
         <v>Roberts1986Pp10to16hDurat21CvSyrian</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
         <v>10</v>
-      </c>
-      <c r="C8" t="s">
-        <v>11</v>
       </c>
       <c r="D8" s="1">
         <v>10</v>
@@ -15149,7 +15149,7 @@
         <v>979.44954128440099</v>
       </c>
       <c r="N8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O8">
         <f t="shared" si="4"/>
@@ -15174,10 +15174,10 @@
         <v>Roberts1986Pp10to16hDurat17CvSyrian</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
         <v>10</v>
-      </c>
-      <c r="C9" t="s">
-        <v>11</v>
       </c>
       <c r="D9" s="1">
         <v>10</v>
@@ -15213,7 +15213,7 @@
         <v>904.58715596330046</v>
       </c>
       <c r="N9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O9">
         <f t="shared" si="4"/>
@@ -15238,10 +15238,10 @@
         <v>Roberts1986Pp10to16hDurat13CvSyrian</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
         <v>10</v>
-      </c>
-      <c r="C10" t="s">
-        <v>11</v>
       </c>
       <c r="D10" s="1">
         <v>10</v>
@@ -15277,7 +15277,7 @@
         <v>792.29357798164858</v>
       </c>
       <c r="N10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O10">
         <f t="shared" si="4"/>
@@ -15302,10 +15302,10 @@
         <v>Roberts1986Pp10to16hDurat9CvSyrian</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
         <v>10</v>
-      </c>
-      <c r="C11" t="s">
-        <v>11</v>
       </c>
       <c r="D11" s="1">
         <v>10</v>
@@ -15341,7 +15341,7 @@
         <v>786.05504587155724</v>
       </c>
       <c r="N11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O11">
         <f t="shared" si="4"/>
@@ -15366,10 +15366,10 @@
         <v>Roberts1986Pp10to16hDurat0CvSyrian</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
         <v>10</v>
-      </c>
-      <c r="C12" t="s">
-        <v>11</v>
       </c>
       <c r="D12" s="1">
         <v>10</v>
@@ -15405,7 +15405,7 @@
         <v>748.62385321100896</v>
       </c>
       <c r="N12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O12">
         <f t="shared" si="4"/>
@@ -15430,10 +15430,10 @@
         <v>Roberts1986Pp16to10hDurat45CvSyrian</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
         <v>10</v>
-      </c>
-      <c r="C13" t="s">
-        <v>11</v>
       </c>
       <c r="D13" s="1">
         <v>16</v>
@@ -15469,7 +15469,7 @@
         <v>723.66972477063985</v>
       </c>
       <c r="N13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O13">
         <f t="shared" si="4"/>
@@ -15494,10 +15494,10 @@
         <v>Roberts1986Pp16to10hDurat41CvSyrian</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
         <v>10</v>
-      </c>
-      <c r="C14" t="s">
-        <v>11</v>
       </c>
       <c r="D14" s="1">
         <v>16</v>
@@ -15533,7 +15533,7 @@
         <v>748.62385321100896</v>
       </c>
       <c r="N14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O14">
         <f t="shared" si="4"/>
@@ -15558,10 +15558,10 @@
         <v>Roberts1986Pp16to10hDurat37CvSyrian</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
         <v>10</v>
-      </c>
-      <c r="C15" t="s">
-        <v>11</v>
       </c>
       <c r="D15" s="1">
         <v>16</v>
@@ -15597,7 +15597,7 @@
         <v>742.38532110091739</v>
       </c>
       <c r="N15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O15">
         <f t="shared" si="4"/>
@@ -15622,10 +15622,10 @@
         <v>Roberts1986Pp16to10hDurat33CvSyrian</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
         <v>10</v>
-      </c>
-      <c r="C16" t="s">
-        <v>11</v>
       </c>
       <c r="D16" s="1">
         <v>16</v>
@@ -15661,7 +15661,7 @@
         <v>748.62385321100896</v>
       </c>
       <c r="N16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O16">
         <f t="shared" si="4"/>
@@ -15686,10 +15686,10 @@
         <v>Roberts1986Pp16to10hDurat29CvSyrian</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" t="s">
         <v>10</v>
-      </c>
-      <c r="C17" t="s">
-        <v>11</v>
       </c>
       <c r="D17" s="1">
         <v>16</v>
@@ -15725,7 +15725,7 @@
         <v>765</v>
       </c>
       <c r="N17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O17">
         <f t="shared" si="4"/>
@@ -15750,10 +15750,10 @@
         <v>Roberts1986Pp16to10hDurat25CvSyrian</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
         <v>10</v>
-      </c>
-      <c r="C18" t="s">
-        <v>11</v>
       </c>
       <c r="D18" s="1">
         <v>16</v>
@@ -15789,7 +15789,7 @@
         <v>754.86238532110019</v>
       </c>
       <c r="N18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O18">
         <f t="shared" si="4"/>
@@ -15814,10 +15814,10 @@
         <v>Roberts1986Pp16to10hDurat21CvSyrian</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" t="s">
         <v>10</v>
-      </c>
-      <c r="C19" t="s">
-        <v>11</v>
       </c>
       <c r="D19" s="1">
         <v>16</v>
@@ -15853,7 +15853,7 @@
         <v>2046.2385321100915</v>
       </c>
       <c r="N19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O19">
         <f t="shared" si="4"/>
@@ -15878,10 +15878,10 @@
         <v>Roberts1986Pp16to10hDurat17CvSyrian</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" t="s">
         <v>10</v>
-      </c>
-      <c r="C20" t="s">
-        <v>11</v>
       </c>
       <c r="D20" s="1">
         <v>16</v>
@@ -15917,7 +15917,7 @@
         <v>2832.2935779816517</v>
       </c>
       <c r="N20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O20">
         <f t="shared" si="4"/>
@@ -15942,10 +15942,10 @@
         <v>Roberts1986Pp16to10hDurat13CvSyrian</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" t="s">
         <v>10</v>
-      </c>
-      <c r="C21" t="s">
-        <v>11</v>
       </c>
       <c r="D21" s="1">
         <v>16</v>
@@ -15981,7 +15981,7 @@
         <v>2944.5871559633006</v>
       </c>
       <c r="N21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O21">
         <f t="shared" si="4"/>
@@ -16006,10 +16006,10 @@
         <v>Roberts1986Pp16to10hDurat9CvSyrian</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" t="s">
         <v>10</v>
-      </c>
-      <c r="C22" t="s">
-        <v>11</v>
       </c>
       <c r="D22" s="1">
         <v>16</v>
@@ -16045,7 +16045,7 @@
         <v>2189.7247706422004</v>
       </c>
       <c r="N22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O22">
         <f t="shared" si="4"/>
@@ -16070,10 +16070,10 @@
         <v>Roberts1986Pp16to10hDurat0CvSyrian</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" t="s">
         <v>10</v>
-      </c>
-      <c r="C23" t="s">
-        <v>11</v>
       </c>
       <c r="D23" s="1">
         <v>16</v>
@@ -16109,7 +16109,7 @@
         <v>2713.7614678899085</v>
       </c>
       <c r="N23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O23">
         <f t="shared" si="4"/>
@@ -16173,7 +16173,7 @@
         <v>1448.4333101074726</v>
       </c>
       <c r="N24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O24">
         <f t="shared" si="4"/>
@@ -16237,7 +16237,7 @@
         <v>1293.0549397183331</v>
       </c>
       <c r="N25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O25">
         <f t="shared" si="4"/>
@@ -16301,7 +16301,7 @@
         <v>1289.8872490023416</v>
       </c>
       <c r="N26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O26">
         <f t="shared" si="4"/>
@@ -16365,7 +16365,7 @@
         <v>1226.8834061780783</v>
       </c>
       <c r="N27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="O27">
         <f t="shared" si="4"/>
@@ -16429,7 +16429,7 @@
         <v>1246.8407550516242</v>
       </c>
       <c r="N28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="O28">
         <f t="shared" si="4"/>
@@ -16493,7 +16493,7 @@
         <v>1234.4481746584738</v>
       </c>
       <c r="N29" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O29">
         <f t="shared" si="4"/>
@@ -16557,7 +16557,7 @@
         <v>1175.805515086251</v>
       </c>
       <c r="N30" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O30">
         <f t="shared" si="4"/>
@@ -16621,7 +16621,7 @@
         <v>1186.4751588860031</v>
       </c>
       <c r="N31" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O31">
         <f t="shared" si="4"/>
@@ -16685,7 +16685,7 @@
         <v>1151.0831696965845</v>
       </c>
       <c r="N32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O32">
         <f t="shared" si="4"/>
@@ -16749,7 +16749,7 @@
         <v>1170.9148877768614</v>
       </c>
       <c r="N33" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O33">
         <f t="shared" si="4"/>
@@ -16813,7 +16813,7 @@
         <v>1144.7477882646058</v>
       </c>
       <c r="N34" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O34">
         <f t="shared" si="4"/>
@@ -16877,7 +16877,7 @@
         <v>1187.7045459344179</v>
       </c>
       <c r="N35" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O35">
         <f t="shared" si="4"/>
@@ -16941,7 +16941,7 @@
         <v>1161.4746310255266</v>
       </c>
       <c r="N36" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O36">
         <f t="shared" si="4"/>
@@ -17005,7 +17005,7 @@
         <v>1453.5034099786728</v>
       </c>
       <c r="N37" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O37">
         <f t="shared" si="4"/>
@@ -17069,7 +17069,7 @@
         <v>1676.4711471463841</v>
       </c>
       <c r="N38" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O38">
         <f t="shared" si="4"/>
@@ -17133,7 +17133,7 @@
         <v>1354.9819471717219</v>
       </c>
       <c r="N39" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O39">
         <f t="shared" si="4"/>
@@ -17197,7 +17197,7 @@
         <v>1997.5565338569704</v>
       </c>
       <c r="N40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O40">
         <f t="shared" si="4"/>
@@ -17261,7 +17261,7 @@
         <v>1929.8146154008555</v>
       </c>
       <c r="N41" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O41">
         <f t="shared" si="4"/>
@@ -17325,7 +17325,7 @@
         <v>2143.4946474947692</v>
       </c>
       <c r="N42" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O42">
         <f t="shared" si="4"/>
@@ -17389,7 +17389,7 @@
         <v>2463.3865416692888</v>
       </c>
       <c r="N43" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O43">
         <f t="shared" si="4"/>
@@ -17453,7 +17453,7 @@
         <v>2229.4709782310288</v>
       </c>
       <c r="N44" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O44">
         <f t="shared" si="4"/>
@@ -17517,7 +17517,7 @@
         <v>1861.8573298705689</v>
       </c>
       <c r="N45" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O45">
         <f t="shared" si="4"/>
@@ -17581,7 +17581,7 @@
         <v>1120.5163142213498</v>
       </c>
       <c r="N46" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O46">
         <f t="shared" si="4"/>
@@ -17645,7 +17645,7 @@
         <v>1087.7170990480333</v>
       </c>
       <c r="N47" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O47">
         <f t="shared" si="4"/>
@@ -17709,7 +17709,7 @@
         <v>1140.7764697333041</v>
       </c>
       <c r="N48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O48">
         <f t="shared" si="4"/>
@@ -17773,7 +17773,7 @@
         <v>1095.0984666811999</v>
       </c>
       <c r="N49" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="O49">
         <f t="shared" si="4"/>
@@ -17837,7 +17837,7 @@
         <v>1058.0680909817593</v>
       </c>
       <c r="N50" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="O50">
         <f t="shared" si="4"/>
@@ -17901,7 +17901,7 @@
         <v>986.6942809388845</v>
       </c>
       <c r="N51" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O51">
         <f t="shared" si="4"/>
@@ -17965,7 +17965,7 @@
         <v>962.48092435142655</v>
       </c>
       <c r="N52" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O52">
         <f t="shared" si="4"/>
@@ -18029,7 +18029,7 @@
         <v>912.32468570598076</v>
       </c>
       <c r="N53" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O53">
         <f t="shared" si="4"/>
@@ -18093,7 +18093,7 @@
         <v>871.00138071361073</v>
       </c>
       <c r="N54" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O54">
         <f t="shared" si="4"/>
@@ -18157,7 +18157,7 @@
         <v>838.38747184070905</v>
       </c>
       <c r="N55" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O55">
         <f t="shared" si="4"/>
@@ -18221,7 +18221,7 @@
         <v>839.86992224402172</v>
       </c>
       <c r="N56" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O56">
         <f t="shared" si="4"/>
@@ -18285,7 +18285,7 @@
         <v>858.46232105224874</v>
       </c>
       <c r="N57" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O57">
         <f t="shared" si="4"/>
@@ -18349,7 +18349,7 @@
         <v>851.54421917011757</v>
       </c>
       <c r="N58" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O58">
         <f t="shared" si="4"/>
@@ -18413,7 +18413,7 @@
         <v>861.6742969260938</v>
       </c>
       <c r="N59" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O59">
         <f t="shared" si="4"/>
@@ -18477,7 +18477,7 @@
         <v>824.58215245985025</v>
       </c>
       <c r="N60" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O60">
         <f t="shared" si="4"/>
@@ -18541,7 +18541,7 @@
         <v>890.52031102390652</v>
       </c>
       <c r="N61" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O61">
         <f t="shared" si="4"/>
@@ -18605,7 +18605,7 @@
         <v>952.28907782864565</v>
       </c>
       <c r="N62" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O62">
         <f t="shared" si="4"/>
@@ -18669,7 +18669,7 @@
         <v>966.58854734394129</v>
       </c>
       <c r="N63" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O63">
         <f t="shared" si="4"/>
@@ -18733,7 +18733,7 @@
         <v>1152.7904948768257</v>
       </c>
       <c r="N64" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O64">
         <f t="shared" si="4"/>
@@ -18797,7 +18797,7 @@
         <v>1132.931836349102</v>
       </c>
       <c r="N65" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O65">
         <f t="shared" si="4"/>
@@ -18861,7 +18861,7 @@
         <v>1146.9842307971803</v>
       </c>
       <c r="N66" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O66">
         <f t="shared" si="4"/>
@@ -18925,7 +18925,7 @@
         <v>1161.777850446915</v>
       </c>
       <c r="N67" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O67">
         <f t="shared" ref="O67" si="12">F67*MIN(H67,I67)</f>
@@ -18986,7 +18986,7 @@
         <v>1630.1396322520613</v>
       </c>
       <c r="N68" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="69" spans="1:18" x14ac:dyDescent="0.25">
@@ -19031,7 +19031,7 @@
         <v>1390.0948717140002</v>
       </c>
       <c r="N69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="70" spans="1:18" x14ac:dyDescent="0.25">
@@ -19076,7 +19076,7 @@
         <v>1365.8459653383368</v>
       </c>
       <c r="N70" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="71" spans="1:18" x14ac:dyDescent="0.25">
@@ -19121,7 +19121,7 @@
         <v>1332.9574661347037</v>
       </c>
       <c r="N71" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="72" spans="1:18" x14ac:dyDescent="0.25">
@@ -19166,7 +19166,7 @@
         <v>1235.3245533250265</v>
       </c>
       <c r="N72" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="73" spans="1:18" x14ac:dyDescent="0.25">
@@ -19211,7 +19211,7 @@
         <v>1258.5570387775358</v>
       </c>
       <c r="N73" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="74" spans="1:18" x14ac:dyDescent="0.25">
@@ -19256,7 +19256,7 @@
         <v>1165.2237175342582</v>
       </c>
       <c r="N74" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="75" spans="1:18" x14ac:dyDescent="0.25">
@@ -19301,7 +19301,7 @@
         <v>1115.0721965527555</v>
       </c>
       <c r="N75" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="76" spans="1:18" x14ac:dyDescent="0.25">
@@ -19346,7 +19346,7 @@
         <v>1073.5764322772916</v>
       </c>
       <c r="N76" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="77" spans="1:18" x14ac:dyDescent="0.25">
@@ -19391,7 +19391,7 @@
         <v>1044.9794427010213</v>
       </c>
       <c r="N77" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="78" spans="1:18" x14ac:dyDescent="0.25">
@@ -19436,7 +19436,7 @@
         <v>1082.1769195590789</v>
       </c>
       <c r="N78" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="79" spans="1:18" x14ac:dyDescent="0.25">
@@ -19481,7 +19481,7 @@
         <v>999.3075158090594</v>
       </c>
       <c r="N79" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="80" spans="1:18" x14ac:dyDescent="0.25">
@@ -19526,7 +19526,7 @@
         <v>1024.126448835412</v>
       </c>
       <c r="N80" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.25">
@@ -19571,7 +19571,7 @@
         <v>955.9555438159357</v>
       </c>
       <c r="N81" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.25">
@@ -19616,7 +19616,7 @@
         <v>976.54017788150657</v>
       </c>
       <c r="N82" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.25">
@@ -19661,7 +19661,7 @@
         <v>1015.8631621276385</v>
       </c>
       <c r="N83" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.25">
@@ -19706,7 +19706,7 @@
         <v>1036.4740526390474</v>
       </c>
       <c r="N84" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.25">
@@ -19751,7 +19751,7 @@
         <v>1435.6766357056113</v>
       </c>
       <c r="N85" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.25">
@@ -19796,7 +19796,7 @@
         <v>1493.6767050920153</v>
       </c>
       <c r="N86" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.25">
@@ -19841,7 +19841,7 @@
         <v>1593.7571050100125</v>
       </c>
       <c r="N87" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
@@ -19886,7 +19886,7 @@
         <v>1684.4552016148089</v>
       </c>
       <c r="N88" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
@@ -19931,7 +19931,7 @@
         <v>1789.1917445949557</v>
       </c>
       <c r="N89" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.25">
@@ -19976,7 +19976,7 @@
         <v>1766.9187705990873</v>
       </c>
       <c r="N90" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
@@ -19999,24 +19999,24 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>42</v>
-      </c>
-      <c r="D1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C2">
         <v>0.41868386608424402</v>
@@ -20031,7 +20031,7 @@
         <v>A</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C3">
         <v>45.0506993834071</v>
@@ -20046,7 +20046,7 @@
         <v>A</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C4">
         <v>75.787299134246894</v>
@@ -20055,18 +20055,18 @@
         <v>0.98967877249144398</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5">
         <v>0.19869742797218401</v>
@@ -20075,16 +20075,16 @@
         <v>0.94382066768643602</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
         <v>36</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>37</v>
-      </c>
-      <c r="J5" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -20093,7 +20093,7 @@
         <v>b</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6">
         <v>41.462318452052401</v>
@@ -20102,7 +20102,7 @@
         <v>0.94602053206755699</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H6">
         <v>0.41868386608424402</v>
@@ -20120,7 +20120,7 @@
         <v>b</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7">
         <v>64.409505937268307</v>
@@ -20129,7 +20129,7 @@
         <v>0.94516108684339095</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H7">
         <v>0.19869742797218401</v>
@@ -20143,10 +20143,10 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C8">
         <v>0.189235645687794</v>
@@ -20155,7 +20155,7 @@
         <v>0.89887720183558495</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H8">
         <v>0.189235645687794</v>
@@ -20173,7 +20173,7 @@
         <v>c</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9">
         <v>37.4528882090423</v>
@@ -20182,7 +20182,7 @@
         <v>0.90122687776954202</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H9">
         <v>0.17937962247488601</v>
@@ -20200,7 +20200,7 @@
         <v>c</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10">
         <v>63.558339772601798</v>
@@ -20209,7 +20209,7 @@
         <v>0.90212180467727399</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H10">
         <v>0.38162521880371902</v>
@@ -20223,10 +20223,10 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C11">
         <v>0.17937962247488601</v>
@@ -20235,7 +20235,7 @@
         <v>0.852061091574282</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H11">
         <v>0.37176919559081101</v>
@@ -20253,7 +20253,7 @@
         <v>d</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C12">
         <v>33.442669484175099</v>
@@ -20262,7 +20262,7 @@
         <v>0.85268793465062298</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H12">
         <v>0.151388516550234</v>
@@ -20280,7 +20280,7 @@
         <v>d</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13">
         <v>62.285730055351401</v>
@@ -20289,7 +20289,7 @@
         <v>0.85722564773784504</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H13">
         <v>0.35284563102203398</v>
@@ -20303,10 +20303,10 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C14">
         <v>0.38162521880371902</v>
@@ -20315,7 +20315,7 @@
         <v>0.81272767413621705</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H14">
         <v>0.13325343383848601</v>
@@ -20333,7 +20333,7 @@
         <v>e</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C15">
         <v>29.644552378849699</v>
@@ -20342,7 +20342,7 @@
         <v>0.81163168435494204</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H15">
         <v>0.124185892482614</v>
@@ -20360,7 +20360,7 @@
         <v>e</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C16">
         <v>57.854856259757398</v>
@@ -20369,7 +20369,7 @@
         <v>0.81057511866651899</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H16">
         <v>-9.6194786557962403E-2</v>
@@ -20383,10 +20383,10 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C17">
         <v>0.37176919559081101</v>
@@ -20395,7 +20395,7 @@
         <v>0.76591156387491499</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H17">
         <v>0.105262327913834</v>
@@ -20413,7 +20413,7 @@
         <v>f</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C18">
         <v>25.003548168356598</v>
@@ -20422,7 +20422,7 @@
         <v>0.76686168451263903</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H18">
         <v>0.30553671960008399</v>
@@ -20440,7 +20440,7 @@
         <v>f</v>
       </c>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C19">
         <v>59.319855550123698</v>
@@ -20449,7 +20449,7 @@
         <v>0.76932174790658003</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H19">
         <v>-0.124974374339647</v>
@@ -20463,10 +20463,10 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C20">
         <v>0.151388516550234</v>
@@ -20475,7 +20475,7 @@
         <v>0.71910333843218199</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H20">
         <v>0.28661315503130402</v>
@@ -20493,7 +20493,7 @@
         <v>g</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C21">
         <v>21.4147729960733</v>
@@ -20502,7 +20502,7 @@
         <v>0.72017961616703197</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H21">
         <v>6.7415198776274096E-2</v>
@@ -20520,7 +20520,7 @@
         <v>g</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C22">
         <v>55.098717928500399</v>
@@ -20529,7 +20529,7 @@
         <v>0.71891804519577995</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H22">
         <v>-0.15257123933578101</v>
@@ -20543,10 +20543,10 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C23">
         <v>0.35284563102203398</v>
@@ -20555,7 +20555,7 @@
         <v>0.67602463217321296</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H23">
         <v>-0.162033021620171</v>
@@ -20573,7 +20573,7 @@
         <v>h</v>
       </c>
       <c r="B24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C24">
         <v>18.037705202403199</v>
@@ -20582,7 +20582,7 @@
         <v>0.67910759623421002</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H24">
         <v>-0.17149480390456101</v>
@@ -20600,7 +20600,7 @@
         <v>h</v>
       </c>
       <c r="B25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C25">
         <v>52.984009587939298</v>
@@ -20609,7 +20609,7 @@
         <v>0.67405342753063202</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H25">
         <v>-0.18056234526043699</v>
@@ -20623,10 +20623,10 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B26" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C26">
         <v>0.13325343383848601</v>
@@ -20635,7 +20635,7 @@
         <v>0.63296169555138504</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H26">
         <v>2.0500528282841601E-2</v>
@@ -20653,7 +20653,7 @@
         <v>i</v>
       </c>
       <c r="B27" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C27">
         <v>13.3970952328386</v>
@@ -20662,7 +20662,7 @@
         <v>0.636210240802359</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H27">
         <v>1.14329869269695E-2</v>
@@ -20680,7 +20680,7 @@
         <v>i</v>
       </c>
       <c r="B28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C28">
         <v>51.291533281819099</v>
@@ -20691,10 +20691,10 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C29">
         <v>0.124185892482614</v>
@@ -20709,7 +20709,7 @@
         <v>j</v>
       </c>
       <c r="B30" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C30">
         <v>9.3864822670430303</v>
@@ -20724,7 +20724,7 @@
         <v>j</v>
       </c>
       <c r="B31" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C31">
         <v>50.228265497610799</v>
@@ -20735,10 +20735,10 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B32" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C32">
         <v>-9.6194786557962403E-2</v>
@@ -20753,7 +20753,7 @@
         <v>k</v>
       </c>
       <c r="B33" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C33">
         <v>48.744342642675697</v>
@@ -20768,7 +20768,7 @@
         <v>k</v>
       </c>
       <c r="B34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C34">
         <v>48.746708088246798</v>
@@ -20779,10 +20779,10 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B35" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C35">
         <v>0.105262327913834</v>
@@ -20797,7 +20797,7 @@
         <v>l</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C36">
         <v>45.789112642517999</v>
@@ -20812,7 +20812,7 @@
         <v>l</v>
       </c>
       <c r="B37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C37">
         <v>49.577767965559097</v>
@@ -20823,10 +20823,10 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B38" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C38">
         <v>0.30553671960008399</v>
@@ -20841,7 +20841,7 @@
         <v>m</v>
       </c>
       <c r="B39" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C39">
         <v>41.5695519846088</v>
@@ -20856,7 +20856,7 @@
         <v>m</v>
       </c>
       <c r="B40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C40">
         <v>46.200700171888997</v>
@@ -20867,10 +20867,10 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B41" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C41">
         <v>-0.124974374339647</v>
@@ -20885,7 +20885,7 @@
         <v>n</v>
       </c>
       <c r="B42" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C42">
         <v>37.558544777884599</v>
@@ -20900,7 +20900,7 @@
         <v>n</v>
       </c>
       <c r="B43" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C43">
         <v>46.821629634302099</v>
@@ -20911,10 +20911,10 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B44" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C44">
         <v>0.28661315503130402</v>
@@ -20929,7 +20929,7 @@
         <v>o</v>
       </c>
       <c r="B45" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C45">
         <v>33.340166842760901</v>
@@ -20944,7 +20944,7 @@
         <v>o</v>
       </c>
       <c r="B46" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C46">
         <v>48.286628924668399</v>
@@ -20955,10 +20955,10 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B47" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C47">
         <v>6.7415198776274096E-2</v>
@@ -20973,7 +20973,7 @@
         <v>p</v>
       </c>
       <c r="B48" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C48">
         <v>29.752180152334599</v>
@@ -20988,7 +20988,7 @@
         <v>p</v>
       </c>
       <c r="B49" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C49">
         <v>48.908741109867002</v>
@@ -20999,10 +20999,10 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B50" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C50">
         <v>-0.15257123933578101</v>
@@ -21017,7 +21017,7 @@
         <v>q</v>
       </c>
       <c r="B51" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C51">
         <v>25.5322252534969</v>
@@ -21032,7 +21032,7 @@
         <v>q</v>
       </c>
       <c r="B52" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C52">
         <v>66.5845331398924</v>
@@ -21043,10 +21043,10 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B53" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C53">
         <v>-0.162033021620171</v>
@@ -21061,7 +21061,7 @@
         <v>r</v>
       </c>
       <c r="B54" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C54">
         <v>21.7321369435289</v>
@@ -21076,7 +21076,7 @@
         <v>r</v>
       </c>
       <c r="B55" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C55">
         <v>68.890842571712398</v>
@@ -21087,10 +21087,10 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B56" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C56">
         <v>-0.17149480390456101</v>
@@ -21105,7 +21105,7 @@
         <v>s</v>
       </c>
       <c r="B57" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C57">
         <v>17.934019838203501</v>
@@ -21120,7 +21120,7 @@
         <v>s</v>
       </c>
       <c r="B58" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C58">
         <v>73.092662387838402</v>
@@ -21131,10 +21131,10 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B59" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C59">
         <v>-0.18056234526043699</v>
@@ -21149,7 +21149,7 @@
         <v>t</v>
       </c>
       <c r="B60" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C60">
         <v>13.503540283537999</v>
@@ -21164,7 +21164,7 @@
         <v>t</v>
       </c>
       <c r="B61" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C61">
         <v>76.871855928594996</v>
@@ -21175,10 +21175,10 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B62" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C62">
         <v>2.0500528282841601E-2</v>
@@ -21193,7 +21193,7 @@
         <v>u</v>
       </c>
       <c r="B63" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C63">
         <v>9.4937157995994408</v>
@@ -21208,7 +21208,7 @@
         <v>u</v>
       </c>
       <c r="B64" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C64">
         <v>81.283411918691698</v>
@@ -21219,10 +21219,10 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B65" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C65">
         <v>1.14329869269695E-2</v>
@@ -21237,7 +21237,7 @@
         <v>v</v>
       </c>
       <c r="B66" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C66">
         <v>9.4617822843900898E-3</v>
@@ -21252,7 +21252,7 @@
         <v>v</v>
       </c>
       <c r="B67" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C67">
         <v>79.590935612571499</v>

</xml_diff>